<commit_message>
Practicing graph data struture
</commit_message>
<xml_diff>
--- a/dsa_mastery_roadmap_new.xlsx
+++ b/dsa_mastery_roadmap_new.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="287" uniqueCount="244">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="288" uniqueCount="245">
   <si>
     <t>Sequence ID</t>
   </si>
@@ -348,6 +348,9 @@
   <si>
     <t>Clone Graph (LeetCode 133)
 Number of Islands (LeetCode 200)</t>
+  </si>
+  <si>
+    <t>Recommended learning order: Graph basics → adjacency lists and matrices → BFS and DFS → connected components → cycle detection → shortest-path algorithms such as Dijkstra's algorithm → topological sorting.</t>
   </si>
   <si>
     <t>Advanced Algorithms</t>
@@ -806,10 +809,10 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="4">
+    <numFmt numFmtId="176" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
+    <numFmt numFmtId="42" formatCode="_(&quot;$&quot;* #,##0_);_(&quot;$&quot;* \(#,##0\);_(&quot;$&quot;* &quot;-&quot;_);_(@_)"/>
+    <numFmt numFmtId="177" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="44" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
-    <numFmt numFmtId="42" formatCode="_(&quot;$&quot;* #,##0_);_(&quot;$&quot;* \(#,##0\);_(&quot;$&quot;* &quot;-&quot;_);_(@_)"/>
-    <numFmt numFmtId="176" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
-    <numFmt numFmtId="177" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
   </numFmts>
   <fonts count="23">
     <font>
@@ -838,8 +841,9 @@
       <charset val="134"/>
     </font>
     <font>
+      <u/>
       <sz val="11"/>
-      <color theme="0"/>
+      <color rgb="FF0000FF"/>
       <name val="Calibri"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -854,17 +858,32 @@
     </font>
     <font>
       <sz val="11"/>
-      <color rgb="FFFF0000"/>
+      <color theme="0"/>
       <name val="Calibri"/>
       <charset val="0"/>
       <scheme val="minor"/>
     </font>
     <font>
       <b/>
-      <sz val="18"/>
-      <color theme="3"/>
+      <sz val="11"/>
+      <color rgb="FF3F3F3F"/>
       <name val="Calibri"/>
-      <charset val="134"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF006100"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFA7D00"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -876,15 +895,7 @@
     </font>
     <font>
       <b/>
-      <sz val="11"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="13"/>
+      <sz val="15"/>
       <color theme="3"/>
       <name val="Calibri"/>
       <charset val="134"/>
@@ -900,32 +911,17 @@
     <font>
       <b/>
       <sz val="11"/>
-      <color rgb="FF3F3F3F"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <charset val="0"/>
       <scheme val="minor"/>
     </font>
     <font>
       <b/>
-      <sz val="11"/>
-      <color theme="1"/>
+      <sz val="13"/>
+      <color theme="3"/>
       <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C6500"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
+      <charset val="134"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -937,17 +933,10 @@
     </font>
     <font>
       <b/>
-      <sz val="15"/>
+      <sz val="11"/>
       <color theme="3"/>
       <name val="Calibri"/>
       <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF006100"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -966,6 +955,13 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <u/>
       <sz val="11"/>
       <color rgb="FF800080"/>
@@ -974,15 +970,22 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <u/>
+      <b/>
+      <sz val="18"/>
+      <color theme="3"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <sz val="11"/>
-      <color rgb="FF0000FF"/>
+      <color rgb="FF9C6500"/>
       <name val="Calibri"/>
       <charset val="0"/>
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="36">
+  <fills count="37">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1009,13 +1012,97 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="FF00B050"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFA5A5A5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF2F2F2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC6EFCE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFCC99"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC7CE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor theme="5"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFA5A5A5"/>
+        <fgColor theme="5" tint="0.799981688894314"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1033,7 +1120,25 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.799981688894314"/>
+        <fgColor rgb="FFFFFFCC"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.399975585192419"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1045,79 +1150,25 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFCC99"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFF2F2F2"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFEB9C"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor theme="7" tint="0.599993896298105"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="4"/>
+        <fgColor theme="4" tint="0.599993896298105"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.799981688894314"/>
+        <fgColor theme="8" tint="0.599993896298105"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFC7CE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFC6EFCE"/>
+        <fgColor theme="7" tint="0.399975585192419"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1129,67 +1180,25 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFCC"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor theme="8" tint="0.799981688894314"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor theme="8" tint="0.399975585192419"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.399975585192419"/>
+        <fgColor theme="9" tint="0.599993896298105"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.599993896298105"/>
+        <fgColor rgb="FFFFEB9C"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1233,20 +1242,17 @@
       <diagonal/>
     </border>
     <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color theme="4" tint="0.499984740745262"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color theme="4"/>
+      <left style="thin">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF3F3F3F"/>
       </bottom>
       <diagonal/>
     </border>
@@ -1266,17 +1272,11 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF3F3F3F"/>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="4"/>
       </bottom>
       <diagonal/>
     </border>
@@ -1288,6 +1288,15 @@
       </top>
       <bottom style="double">
         <color theme="4"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="4" tint="0.499984740745262"/>
       </bottom>
       <diagonal/>
     </border>
@@ -1318,152 +1327,152 @@
   </borders>
   <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="15" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="6" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="3" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="28" borderId="9" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="12" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="15" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="10" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="23" borderId="9" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="12" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="8" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="5" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="5" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="177" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="176" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="6" borderId="2" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="6" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1486,6 +1495,7 @@
     <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="49">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1832,8 +1842,8 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:G24"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15" outlineLevelCol="6"/>
+  <dimension ref="A1:H24"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15" outlineLevelCol="7"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="20" customWidth="1"/>
@@ -2235,7 +2245,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="18" ht="42" customHeight="1" spans="1:7">
+    <row r="18" ht="42" customHeight="1" spans="1:8">
       <c r="A18" s="2">
         <v>17</v>
       </c>
@@ -2256,6 +2266,9 @@
       </c>
       <c r="G18" s="6" t="s">
         <v>97</v>
+      </c>
+      <c r="H18" s="8" t="s">
+        <v>98</v>
       </c>
     </row>
     <row r="19" ht="42" customHeight="1" spans="1:7">
@@ -2263,22 +2276,22 @@
         <v>18</v>
       </c>
       <c r="B19" s="4" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="C19" s="5" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="D19" s="7" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="E19" s="7" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="F19" s="4" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="G19" s="7" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
     </row>
     <row r="20" ht="42" customHeight="1" spans="1:7">
@@ -2286,22 +2299,22 @@
         <v>19</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="C20" s="3" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="D20" s="6" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="E20" s="6" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="F20" s="2" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="G20" s="6" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
     </row>
     <row r="21" ht="42" customHeight="1" spans="1:7">
@@ -2309,22 +2322,22 @@
         <v>20</v>
       </c>
       <c r="B21" s="4" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="C21" s="5" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="D21" s="7" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="E21" s="7" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="F21" s="4" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="G21" s="7" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
     </row>
     <row r="22" ht="42" customHeight="1" spans="1:7">
@@ -2332,22 +2345,22 @@
         <v>21</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="C22" s="3" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="D22" s="6" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="E22" s="6" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="F22" s="2" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="G22" s="6" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
     </row>
     <row r="23" ht="42" customHeight="1" spans="1:7">
@@ -2358,19 +2371,19 @@
         <v>82</v>
       </c>
       <c r="C23" s="5" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="D23" s="7" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="E23" s="7" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="F23" s="4" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="G23" s="7" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
     </row>
     <row r="24" ht="42" customHeight="1" spans="1:7">
@@ -2378,22 +2391,22 @@
         <v>23</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="C24" s="3" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="D24" s="6" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="E24" s="6" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="F24" s="2" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="G24" s="6" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
     </row>
   </sheetData>
@@ -2418,22 +2431,22 @@
   <sheetData>
     <row r="1" ht="28" customHeight="1" spans="1:6">
       <c r="A1" s="1" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>1</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
     </row>
     <row r="2" ht="36" customHeight="1" spans="1:6">
@@ -2444,16 +2457,16 @@
         <v>1</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="E2" s="6" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="F2" s="6" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
     </row>
     <row r="3" ht="36" customHeight="1" spans="1:6">
@@ -2464,16 +2477,16 @@
         <v>2</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="D3" s="5" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="E3" s="7" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="F3" s="7" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
     </row>
     <row r="4" ht="36" customHeight="1" spans="1:6">
@@ -2484,16 +2497,16 @@
         <v>3</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="E4" s="6" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="F4" s="6" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
     </row>
     <row r="5" ht="36" customHeight="1" spans="1:6">
@@ -2504,16 +2517,16 @@
         <v>4</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="E5" s="7" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="F5" s="7" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
     </row>
     <row r="6" ht="36" customHeight="1" spans="1:6">
@@ -2524,16 +2537,16 @@
         <v>5</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="E6" s="6" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="F6" s="6" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
     </row>
     <row r="7" ht="36" customHeight="1" spans="1:6">
@@ -2544,16 +2557,16 @@
         <v>6</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="E7" s="7" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="F7" s="7" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
     </row>
     <row r="8" ht="36" customHeight="1" spans="1:6">
@@ -2564,16 +2577,16 @@
         <v>7</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="D8" s="3" t="s">
         <v>45</v>
       </c>
       <c r="E8" s="6" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="F8" s="6" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
     </row>
     <row r="9" ht="36" customHeight="1" spans="1:6">
@@ -2584,16 +2597,16 @@
         <v>8</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="D9" s="5" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="E9" s="7" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="F9" s="7" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="10" ht="36" customHeight="1" spans="1:6">
@@ -2604,16 +2617,16 @@
         <v>9</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="D10" s="3" t="s">
         <v>29</v>
       </c>
       <c r="E10" s="6" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="F10" s="6" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
     </row>
     <row r="11" ht="36" customHeight="1" spans="1:6">
@@ -2624,16 +2637,16 @@
         <v>10</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="D11" s="5" t="s">
         <v>34</v>
       </c>
       <c r="E11" s="7" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="F11" s="7" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
     </row>
     <row r="12" ht="36" customHeight="1" spans="1:6">
@@ -2644,16 +2657,16 @@
         <v>11</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="D12" s="3" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="E12" s="6" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="F12" s="6" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
     </row>
     <row r="13" ht="36" customHeight="1" spans="1:6">
@@ -2664,16 +2677,16 @@
         <v>12</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="D13" s="5" t="s">
         <v>72</v>
       </c>
       <c r="E13" s="7" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="F13" s="7" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
     </row>
     <row r="14" ht="36" customHeight="1" spans="1:6">
@@ -2684,16 +2697,16 @@
         <v>13</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="D14" s="3" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="E14" s="6" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="F14" s="6" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
     </row>
     <row r="15" ht="36" customHeight="1" spans="1:6">
@@ -2704,16 +2717,16 @@
         <v>14</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="D15" s="5" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="E15" s="7" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="F15" s="7" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
     </row>
     <row r="16" ht="36" customHeight="1" spans="1:6">
@@ -2724,16 +2737,16 @@
         <v>15</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="D16" s="3" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="E16" s="6" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="F16" s="6" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
     </row>
     <row r="17" ht="36" customHeight="1" spans="1:6">
@@ -2744,16 +2757,16 @@
         <v>16</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="D17" s="5" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="E17" s="7" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="F17" s="7" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
     </row>
     <row r="18" ht="36" customHeight="1" spans="1:6">
@@ -2764,16 +2777,16 @@
         <v>17</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="D18" s="3" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="E18" s="6" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="F18" s="6" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
     </row>
     <row r="19" ht="36" customHeight="1" spans="1:6">
@@ -2784,16 +2797,16 @@
         <v>18</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="D19" s="5" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="E19" s="7" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="F19" s="7" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
     </row>
     <row r="20" ht="36" customHeight="1" spans="1:6">
@@ -2804,16 +2817,16 @@
         <v>19</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="D20" s="3" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="E20" s="6" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="F20" s="6" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
     </row>
     <row r="21" ht="36" customHeight="1" spans="1:6">
@@ -2824,16 +2837,16 @@
         <v>20</v>
       </c>
       <c r="C21" s="4" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="D21" s="5" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="E21" s="7" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="F21" s="7" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
     </row>
     <row r="22" ht="36" customHeight="1" spans="1:6">
@@ -2844,16 +2857,16 @@
         <v>21</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="D22" s="3" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="E22" s="6" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="F22" s="6" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
     </row>
     <row r="23" ht="36" customHeight="1" spans="1:6">
@@ -2864,16 +2877,16 @@
         <v>22</v>
       </c>
       <c r="C23" s="4" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="D23" s="5" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="E23" s="7" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="F23" s="7" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
     </row>
     <row r="24" ht="36" customHeight="1" spans="1:6">
@@ -2884,16 +2897,16 @@
         <v>23</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="D24" s="3" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="E24" s="6" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="F24" s="6" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
     </row>
     <row r="25" ht="36" customHeight="1" spans="1:6">
@@ -2904,16 +2917,16 @@
         <v>24</v>
       </c>
       <c r="C25" s="4" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="D25" s="5" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="E25" s="7" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="F25" s="7" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
     </row>
     <row r="26" ht="36" customHeight="1" spans="1:6">
@@ -2924,16 +2937,16 @@
         <v>25</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="D26" s="3" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="E26" s="6" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="F26" s="6" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
     </row>
     <row r="27" ht="36" customHeight="1" spans="1:6">
@@ -2944,16 +2957,16 @@
         <v>26</v>
       </c>
       <c r="C27" s="4" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="D27" s="5" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="E27" s="7" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="F27" s="7" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
     </row>
     <row r="28" ht="36" customHeight="1" spans="1:6">
@@ -2964,16 +2977,16 @@
         <v>27</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="D28" s="3" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="E28" s="6" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="F28" s="6" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
     </row>
     <row r="29" ht="36" customHeight="1" spans="1:6">
@@ -2984,16 +2997,16 @@
         <v>28</v>
       </c>
       <c r="C29" s="4" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="D29" s="5" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="E29" s="7" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="F29" s="7" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
     </row>
     <row r="30" ht="36" customHeight="1" spans="1:6">
@@ -3004,16 +3017,16 @@
         <v>29</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="D30" s="3" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="E30" s="6" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="F30" s="6" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
     </row>
     <row r="31" ht="36" customHeight="1" spans="1:6">
@@ -3024,16 +3037,16 @@
         <v>30</v>
       </c>
       <c r="C31" s="4" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="D31" s="5" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="E31" s="7" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="F31" s="7" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
     </row>
     <row r="32" ht="36" customHeight="1" spans="1:6">
@@ -3044,16 +3057,16 @@
         <v>31</v>
       </c>
       <c r="C32" s="2" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="D32" s="3" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="E32" s="6" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="F32" s="6" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
     </row>
     <row r="33" ht="36" customHeight="1" spans="1:6">
@@ -3064,16 +3077,16 @@
         <v>32</v>
       </c>
       <c r="C33" s="4" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="D33" s="5" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="E33" s="7" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="F33" s="7" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
     </row>
     <row r="34" ht="36" customHeight="1" spans="1:6">
@@ -3084,16 +3097,16 @@
         <v>33</v>
       </c>
       <c r="C34" s="2" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="D34" s="3" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="E34" s="6" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="F34" s="6" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
     </row>
     <row r="35" ht="36" customHeight="1" spans="1:6">
@@ -3104,16 +3117,16 @@
         <v>34</v>
       </c>
       <c r="C35" s="4" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="D35" s="5" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="E35" s="7" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="F35" s="7" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
     </row>
   </sheetData>

</xml_diff>